<commit_message>
Beta feedback round (APickering) and app-wide em dash removal
Feedback fixes: sticky compacting navbar, statistical glossary on the
Definitions tab, distribution/param_type edit validation with snap-back,
double-click wording, MoE defined at first use, grey tornado bars
explained, IPCC Inventory Software note and Word-summary blurb on the
IPCC Report tab, reproducibility note on Simulate, corrected tab
numbering (6 Sensitivity / 7 IPCC Report), QA/QC "where to document"
wording.

Em dashes removed everywhere per style rule (UI strings EN/FR, template
guides, exports, translator prompts, doc sources incl. pandoc --- / --
forms, defaults CSVs, comments); paired-dash asides repaired by hand.
Rebuilt: methodology + user guide (pdf/docx), help pages, translator
kit, feedback guide, blank feedback template. Audit 120/120.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/beta_test/beta_feedback_template.xlsx
+++ b/documentation/beta_test/beta_feedback_template.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
-    <t xml:space="preserve">IPCC Tier 2 Livestock GHG Uncertainty Calculator — Beta Testing Feedback Form</t>
+    <t xml:space="preserve">IPCC Tier 2 Livestock GHG Uncertainty Calculator: Beta Testing Feedback Form</t>
   </si>
   <si>
     <t xml:space="preserve"/>
@@ -31,16 +31,16 @@
     <t xml:space="preserve">2. Use the Type dropdown to classify your comment:</t>
   </si>
   <si>
-    <t xml:space="preserve">   Bug          — the tool crashes, produces wrong numbers, or behaves unexpectedly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Correction   — something is factually incorrect (method, equation, reference) or not IPCC-compliant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Enhancement  — a feature that would make the tool more useful</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   General      — a general comment or question, or feedback from user experience such as a challenge that you were later able to overcome</t>
+    <t xml:space="preserve">   Bug         : the tool crashes, produces wrong numbers, or behaves unexpectedly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Correction  : something is factually incorrect (method, equation, reference) or not IPCC-compliant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Enhancement : a feature that would make the tool more useful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   General     : a general comment or question, or feedback from user experience such as a challenge that you were later able to overcome</t>
   </si>
   <si>
     <t xml:space="preserve">3. Use Severity to indicate urgency (Critical = must fix before release).</t>
@@ -52,37 +52,37 @@
     <t xml:space="preserve">5. Save your completed file and email it to m.lolita@cgiar.org.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Multiple reviewers: combine sheets by appending rows — the Reviewer name column keeps them distinct.</t>
+    <t xml:space="preserve">6. Multiple reviewers: combine sheets by appending rows, the Reviewer name column keeps them distinct.</t>
   </si>
   <si>
     <t xml:space="preserve">COLUMN DEFINITIONS</t>
   </si>
   <si>
-    <t xml:space="preserve">Reviewer name   — Your full name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date            — Date of the observation (YYYY-MM-DD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab             — Which app tab (Home, Definitions, Resources, Data Input, QA/QC, Uncertainty, Correlations, Simulate, Sensitivity, IPCC Report, Contact)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screen element  — The specific button, table, chart, or text that the comment relates to</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type            — Bug / Correction / Enhancement / General</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Severity        — Critical / High / Medium / Low</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description     — What you observed or what the problem is</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suggested fix   — What the correct behaviour should be, or your proposed solution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status          — Leave blank; will be filled by the development team</t>
+    <t xml:space="preserve">Reviewer name  : Your full name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date           : Date of the observation (YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab            : Which app tab (Home, Definitions, Resources, Data Input, QA/QC, Uncertainty, Correlations, Simulate, Sensitivity, IPCC Report, Contact)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen element : The specific button, table, chart, or text that the comment relates to</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type           : Bug / Correction / Enhancement / General</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Severity       : Critical / High / Medium / Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description    : What you observed or what the problem is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suggested fix  : What the correct behaviour should be, or your proposed solution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status         : Leave blank; will be filled by the development team</t>
   </si>
   <si>
     <t xml:space="preserve">Reviewer name</t>
@@ -127,19 +127,19 @@
     <t xml:space="preserve">Critical</t>
   </si>
   <si>
-    <t xml:space="preserve">Must fix before any external release — calculation error or crash</t>
+    <t xml:space="preserve">Must fix before any external release: calculation error or crash</t>
   </si>
   <si>
     <t xml:space="preserve">Correction</t>
   </si>
   <si>
-    <t xml:space="preserve">Something is factually incorrect — wrong equation, wrong IPCC reference, wrong number</t>
+    <t xml:space="preserve">Something is factually incorrect: wrong equation, wrong IPCC reference, wrong number</t>
   </si>
   <si>
     <t xml:space="preserve">High</t>
   </si>
   <si>
-    <t xml:space="preserve">Should fix before external release — significant usability or accuracy issue</t>
+    <t xml:space="preserve">Should fix before external release: significant usability or accuracy issue</t>
   </si>
   <si>
     <t xml:space="preserve">Enhancement</t>
@@ -151,7 +151,7 @@
     <t xml:space="preserve">Medium</t>
   </si>
   <si>
-    <t xml:space="preserve">Can fix in next iteration — minor issue that does not block use</t>
+    <t xml:space="preserve">Can fix in next iteration: minor issue that does not block use</t>
   </si>
   <si>
     <t xml:space="preserve">General</t>
@@ -163,7 +163,7 @@
     <t xml:space="preserve">Low</t>
   </si>
   <si>
-    <t xml:space="preserve">Nice to have — cosmetic or very minor improvement</t>
+    <t xml:space="preserve">Nice to have: cosmetic or very minor improvement</t>
   </si>
 </sst>
 </file>
@@ -1353,13 +1353,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD39130D-D0D9-4720-B59B-9C8CC9732B41}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E452305-83B9-42E7-A630-A95A8360665B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33E9C772-98CC-4F29-8777-B4F511B81E4E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08FF7278-0E7C-432A-AD4E-AD4EC014B1FF}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5FBBEF64-0AD5-49BA-A6A9-0DF7140CABF4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5ADE79DF-6D2A-4EF7-8D3C-EB459B696D26}"/>
 </file>
</xml_diff>